<commit_message>
feat(test): expand Sprint 4 automation test suite to 54 test cases and update Excel report
</commit_message>
<xml_diff>
--- a/Bao_Cao_Kiem_Thu_Sprint4_Le_Quang_Hung.xlsx
+++ b/Bao_Cao_Kiem_Thu_Sprint4_Le_Quang_Hung.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Tổng Quan Sprint 4" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chi Tiết 28 Test Cases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chi Tiết 54 Test Cases" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Báo Cáo Lỗi &amp; Đề Xuất" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -643,7 +643,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>54</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>54</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -788,12 +788,12 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Hoàn thành 100%, bảo mật phân quyền cá nhân, lọc chưa đọc và đánh dấu đã đọc chuẩn xác</t>
+          <t>Hoàn thành 100%, bảo mật phân quyền cá nhân, lọc chưa đọc, idempotency và đánh dấu đã đọc chuẩn xác</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>22</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -872,12 +872,12 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>18</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -902,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -975,7 +975,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
@@ -991,12 +991,12 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>Là thực tập sinh, nhận thông báo ứng dụng để không bỏ lỡ lịch trình</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E2" s="13" t="inlineStr">
         <is>
-          <t>Kiểm tra truy cập xem danh sách thông báo khi chưa đăng nhập / không có token</t>
+          <t>Chưa đăng nhập truy cập xem thông báo</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
@@ -1006,14 +1006,12 @@
       </c>
       <c r="G2" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/notifications/my
-(Header: Không truyền Authorization token)</t>
+          <t>GET /api/v1/notifications/my (Không Bearer Token)</t>
         </is>
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Status 401 Unauthorized
-Detail: 'Không thể xác thực thông tin đăng nhập'</t>
+          <t>Status 401 Unauthorized</t>
         </is>
       </c>
       <c r="I2" s="13" t="inlineStr">
@@ -1028,7 +1026,7 @@
       </c>
       <c r="K2" s="12" t="inlineStr"/>
     </row>
-    <row r="3" ht="45" customHeight="1">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="12" t="n">
         <v>2</v>
       </c>
@@ -1044,35 +1042,32 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Là thực tập sinh, nhận thông báo ứng dụng để không bỏ lỡ lịch trình</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>Kiểm tra người dùng chỉ xem đúng thông báo của mình, không lộ thông báo của người khác</t>
+          <t>Hỗ trợ truy vấn thông báo qua header mock X-User-Id</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/notifications/my
-(Header: Bearer token của User 1)</t>
+          <t>GET /api/v1/notifications/my (Header X-User-Id: 1020)</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Danh sách chỉ chứa thông báo của User 1 (ma_nguoi_nhan == user1.id)
-Đầy đủ total, unread_count, items</t>
+          <t>Status 200 OK, trả về items</t>
         </is>
       </c>
       <c r="I3" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, phân lập dữ liệu chính xác 100%, không lộ dữ liệu User 2</t>
+          <t>HTTP 200 OK hỗ trợ mock header linh hoạt</t>
         </is>
       </c>
       <c r="J3" s="14" t="inlineStr">
@@ -1082,7 +1077,7 @@
       </c>
       <c r="K3" s="12" t="inlineStr"/>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="12" t="n">
         <v>3</v>
       </c>
@@ -1098,34 +1093,32 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Là thực tập sinh, nhận thông báo ứng dụng để không bỏ lỡ lịch trình</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>Kiểm tra bộ lọc chỉ lấy các thông báo chưa đọc (unread_only=true)</t>
+          <t>Người dùng chỉ xem đúng thông báo của mình, không lộ người khác</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Data Isolation</t>
         </is>
       </c>
       <c r="G4" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/notifications/my?unread_only=true
-(Header: Bearer token của User 1)</t>
+          <t>GET /api/v1/notifications/my (Token User 1)</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Danh sách items chỉ chứa bản ghi có da_doc = False</t>
+          <t>Status 200 OK, chỉ trả về thông báo của User 1 (total=2)</t>
         </is>
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, lọc đúng 100% các thông báo chưa đọc</t>
+          <t>HTTP 200 OK phân lập dữ liệu người dùng tuyệt đối</t>
         </is>
       </c>
       <c r="J4" s="14" t="inlineStr">
@@ -1135,7 +1128,7 @@
       </c>
       <c r="K4" s="12" t="inlineStr"/>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="12" t="n">
         <v>4</v>
       </c>
@@ -1151,34 +1144,32 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Là thực tập sinh, nhận thông báo ứng dụng để không bỏ lỡ lịch trình</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Cập nhật trạng thái thông báo thành đã đọc thành công</t>
+          <t>Kiểm tra schema và kiểu dữ liệu trả về của thông báo</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Schema Validation</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/notifications/{id}/read
-(Header: Bearer token chính chủ User 1)</t>
+          <t>GET /api/v1/notifications/my (Token User 1)</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Trường da_doc chuyển sang True trong response và cập nhật vào DB</t>
+          <t>Đầy đủ ma_thong_bao, ma_nguoi_nhan, tieu_de, noi_dung, da_doc</t>
         </is>
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, cập nhật trạng thái đã đọc thành công</t>
+          <t>HTTP 200 OK đúng kiểu dữ liệu mô tả</t>
         </is>
       </c>
       <c r="J5" s="14" t="inlineStr">
@@ -1188,7 +1179,7 @@
       </c>
       <c r="K5" s="12" t="inlineStr"/>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="12" t="n">
         <v>5</v>
       </c>
@@ -1204,34 +1195,32 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Là thực tập sinh, nhận thông báo ứng dụng để không bỏ lỡ lịch trình</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Bắt lỗi khi cập nhật mã thông báo không tồn tại trong hệ thống</t>
+          <t>Bộ lọc unread_only=True chỉ trả về thông báo chưa đọc</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/notifications/999999/read
-(Header: Bearer token User 1)</t>
+          <t>GET /api/v1/notifications/my?unread_only=true</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Status 404 Not Found
-Detail: 'Không tìm thấy thông báo với mã 999999'</t>
+          <t>Status 200 OK, tất cả items có da_doc=False</t>
         </is>
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>HTTP 404 Not Found đúng chuẩn thiết kế REST API</t>
+          <t>HTTP 200 OK lọc đúng thông báo chưa đọc</t>
         </is>
       </c>
       <c r="J6" s="14" t="inlineStr">
@@ -1241,7 +1230,7 @@
       </c>
       <c r="K6" s="12" t="inlineStr"/>
     </row>
-    <row r="7" ht="45" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="12" t="n">
         <v>6</v>
       </c>
@@ -1257,34 +1246,32 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Là thực tập sinh, nhận thông báo ứng dụng để không bỏ lỡ lịch trình</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Bắt lỗi khi người dùng cố tình cập nhật thông báo của người khác</t>
+          <t>Phân trang danh sách thông báo với skip và limit</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/notifications/{id_user2}/read
-(Dùng token của User 1 để sửa thông báo User 2)</t>
+          <t>GET /api/v1/notifications/my?skip=1&amp;limit=2 (5 thông báo)</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Status 403 Forbidden
-Detail: 'Bạn không có quyền truy cập hoặc chỉnh sửa thông báo này'</t>
+          <t>Status 200 OK, items có 2 phần tử, skip=1, limit=2, total=5</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>HTTP 403 Forbidden chặn hành vi truy cập trái phép</t>
+          <t>HTTP 200 OK phân trang thông báo chuẩn xác</t>
         </is>
       </c>
       <c r="J7" s="14" t="inlineStr">
@@ -1294,7 +1281,7 @@
       </c>
       <c r="K7" s="12" t="inlineStr"/>
     </row>
-    <row r="8" ht="45" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="12" t="n">
         <v>7</v>
       </c>
@@ -1310,34 +1297,32 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Là thực tập sinh, nhận thông báo ứng dụng để không bỏ lỡ lịch trình</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>Tiện ích đánh dấu tất cả thông báo cá nhân là đã đọc (read-all)</t>
+          <t>Sắp xếp thông báo theo thời gian tạo mới nhất (ngay_tao DESC)</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/notifications/read-all
-(Header: Bearer token User 1 có 3 thông báo chưa đọc)</t>
+          <t>GET /api/v1/notifications/my (gồm bản ghi cũ và mới)</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-success=True, updated_count &gt;= 3, unread_count chuyển về 0</t>
+          <t>Status 200 OK, thông báo mới nhất đứng đầu danh sách</t>
         </is>
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, toàn bộ thông báo của user chuyển sang đã đọc</t>
+          <t>HTTP 200 OK sắp xếp thời gian giảm dần chuẩn</t>
         </is>
       </c>
       <c r="J8" s="14" t="inlineStr">
@@ -1347,28 +1332,28 @@
       </c>
       <c r="K8" s="12" t="inlineStr"/>
     </row>
-    <row r="9" ht="45" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="12" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>TC-AdminUser</t>
+          <t>TC-Notification</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_01</t>
+          <t>TC_NTF_08</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Admin tạo tài khoản người dùng vai trò Admin thành công</t>
+          <t>Cập nhật trạng thái thông báo thành đã đọc thành công</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -1378,25 +1363,17 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-{
-  'ten_dang_nhap': 'user_test_admin_2026',
-  'email': 'admin.sprint4@company.com',
-  'mat_khau': 'MatKhauChuan@123',
-  'ho_ten': 'Người Dùng Admin',
-  'vai_tro': 'Admin'
-}</t>
+          <t>PATCH /api/v1/notifications/{id}/read (Token chính chủ)</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Status 201 Created
-Trả về đầy đủ ten_dang_nhap, email, vai_tro='Admin', trang_thai=True</t>
+          <t>Status 200 OK, da_doc chuyển thành True trong DB và response</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>HTTP 201 Created, tạo tài khoản Admin thành công</t>
+          <t>HTTP 200 OK cập nhật trạng thái đã đọc thành công</t>
         </is>
       </c>
       <c r="J9" s="14" t="inlineStr">
@@ -1406,28 +1383,28 @@
       </c>
       <c r="K9" s="12" t="inlineStr"/>
     </row>
-    <row r="10" ht="45" customHeight="1">
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="12" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>TC-AdminUser</t>
+          <t>TC-Notification</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_02</t>
+          <t>TC_NTF_09</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Admin tạo tài khoản người dùng vai trò HR thành công</t>
+          <t>Đánh dấu đã đọc lại thông báo đã đọc trước đó (Idempotency)</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
@@ -1437,25 +1414,17 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-{
-  'ten_dang_nhap': 'user_test_hr_2026',
-  'email': 'hr.sprint4@company.com',
-  'mat_khau': 'MatKhauChuan@123',
-  'ho_ten': 'Người Dùng HR',
-  'vai_tro': 'HR'
-}</t>
+          <t>PATCH /api/v1/notifications/{id}/read (Đã đọc trước đó)</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Status 201 Created
-Trả về đầy đủ ten_dang_nhap, email, vai_tro='HR', trang_thai=True</t>
+          <t>Status 200 OK, da_doc tiếp tục duy trì True mà không lỗi</t>
         </is>
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>HTTP 201 Created, tạo tài khoản HR thành công</t>
+          <t>HTTP 200 OK tính lũy thừa idempotent an toàn</t>
         </is>
       </c>
       <c r="J10" s="14" t="inlineStr">
@@ -1465,56 +1434,48 @@
       </c>
       <c r="K10" s="12" t="inlineStr"/>
     </row>
-    <row r="11" ht="45" customHeight="1">
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="12" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>TC-AdminUser</t>
+          <t>TC-Notification</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_03</t>
+          <t>TC_NTF_10</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Admin tạo tài khoản người dùng vai trò Mentor thành công</t>
+          <t>Bắt lỗi khi cập nhật mã thông báo không tồn tại</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-{
-  'ten_dang_nhap': 'user_test_mentor_2026',
-  'email': 'mentor.sprint4@company.com',
-  'mat_khau': 'MatKhauChuan@123',
-  'ho_ten': 'Người Dùng Mentor',
-  'vai_tro': 'Mentor'
-}</t>
+          <t>PATCH /api/v1/notifications/999999/read</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Status 201 Created
-Trả về đầy đủ ten_dang_nhap, email, vai_tro='Mentor', trang_thai=True</t>
+          <t>Status 404 Not Found, detail: 'Không tìm thấy thông báo'</t>
         </is>
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>HTTP 201 Created, tạo tài khoản Mentor thành công</t>
+          <t>HTTP 404 Not Found đúng chuẩn REST API</t>
         </is>
       </c>
       <c r="J11" s="14" t="inlineStr">
@@ -1524,56 +1485,48 @@
       </c>
       <c r="K11" s="12" t="inlineStr"/>
     </row>
-    <row r="12" ht="45" customHeight="1">
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" s="12" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>TC-AdminUser</t>
+          <t>TC-Notification</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_04</t>
+          <t>TC_NTF_11</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>Admin tạo tài khoản người dùng vai trò ThucTapSinh thành công</t>
+          <t>Chặn người dùng cập nhật thông báo của người khác</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-{
-  'ten_dang_nhap': 'user_test_tts_2026',
-  'email': 'tts.sprint4@company.com',
-  'mat_khau': 'MatKhauChuan@123',
-  'ho_ten': 'Người Dùng Thực Tập Sinh',
-  'vai_tro': 'ThucTapSinh'
-}</t>
+          <t>PATCH /api/v1/notifications/{id_user2}/read (Token User 1)</t>
         </is>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Status 201 Created
-Trả về đầy đủ ten_dang_nhap, email, vai_tro='ThucTapSinh', trang_thai=True</t>
+          <t>Status 403 Forbidden, detail: 'Bạn không có quyền'</t>
         </is>
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>HTTP 201 Created, tạo tài khoản Thực tập sinh thành công</t>
+          <t>HTTP 403 Forbidden bảo vệ quyền riêng tư</t>
         </is>
       </c>
       <c r="J12" s="14" t="inlineStr">
@@ -1583,52 +1536,48 @@
       </c>
       <c r="K12" s="12" t="inlineStr"/>
     </row>
-    <row r="13" ht="45" customHeight="1">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="12" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>TC-AdminUser</t>
+          <t>TC-Notification</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_05</t>
+          <t>TC_NTF_12</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Mật khẩu được băm an toàn bằng bcrypt trong DB và không lộ trong response</t>
+          <t>Tiện ích đánh dấu tất cả thông báo cá nhân là đã đọc (read-all)</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-Payload mang mật khẩu thô: 'MatKhauBaoMatTuyetDoi@2026'</t>
+          <t>PATCH /api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Status 201 Created
-1) Response KHÔNG chứa mat_khau, password
-2) DB lưu chuỗi bcrypt hash ($2b$)
-3) verify_password khớp 100%</t>
+          <t>Status 200 OK, success=True, unread_count trở về 0</t>
         </is>
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>HTTP 201 Created, bảo mật mật khẩu an toàn tuyệt đối theo tiêu chuẩn bcrypt</t>
+          <t>HTTP 200 OK cập nhật hàng loạt thành công</t>
         </is>
       </c>
       <c r="J13" s="14" t="inlineStr">
@@ -1638,50 +1587,48 @@
       </c>
       <c r="K13" s="12" t="inlineStr"/>
     </row>
-    <row r="14" ht="45" customHeight="1">
+    <row r="14" ht="42" customHeight="1">
       <c r="A14" s="12" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>TC-AdminUser</t>
+          <t>TC-Notification</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_06</t>
+          <t>TC_NTF_13</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Bắt lỗi chống trùng lặp tên đăng nhập (username)</t>
+          <t>Tạo thông báo mới qua endpoint nội bộ POST /api/v1/notifications</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-Payload mang ten_dang_nhap đã tồn tại trong DB</t>
+          <t>POST /api/v1/notifications {ma_nguoi_nhan, tieu_de, noi_dung, loai_thong_bao}</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Status 400 Bad Request (hoặc 409 Conflict)
-Detail: 'Tên đăng nhập ... đã tồn tại trong hệ thống'</t>
+          <t>Status 201 Created, tạo thông báo mới thành công</t>
         </is>
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>HTTP 400 Bad Request kèm thông báo lỗi trùng lặp rõ ràng</t>
+          <t>HTTP 201 Created chèn thông báo thành công</t>
         </is>
       </c>
       <c r="J14" s="14" t="inlineStr">
@@ -1691,28 +1638,28 @@
       </c>
       <c r="K14" s="12" t="inlineStr"/>
     </row>
-    <row r="15" ht="45" customHeight="1">
+    <row r="15" ht="42" customHeight="1">
       <c r="A15" s="12" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>TC-AdminUser</t>
+          <t>TC-Notification</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_07</t>
+          <t>TC_NTF_14</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là thực tập sinh, nhận thông báo ứng dụng</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Bắt lỗi chống trùng lặp địa chỉ email</t>
+          <t>Bắt lỗi khi truyền mã thông báo không hợp lệ (số &lt;= 0)</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -1722,19 +1669,17 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-Payload mang email đã tồn tại trong DB</t>
+          <t>PATCH /api/v1/notifications/0/read</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>Status 400 Bad Request (hoặc 409 Conflict)
-Detail: 'Email ... đã tồn tại trong hệ thống'</t>
+          <t>Status 422 Unprocessable Entity</t>
         </is>
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>HTTP 400 Bad Request kèm thông báo lỗi trùng lặp rõ ràng</t>
+          <t>HTTP 422 Unprocessable Entity từ FastAPI Path validation</t>
         </is>
       </c>
       <c r="J15" s="14" t="inlineStr">
@@ -1744,7 +1689,7 @@
       </c>
       <c r="K15" s="12" t="inlineStr"/>
     </row>
-    <row r="16" ht="45" customHeight="1">
+    <row r="16" ht="42" customHeight="1">
       <c r="A16" s="12" t="n">
         <v>15</v>
       </c>
@@ -1755,38 +1700,37 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_08</t>
+          <t>TC_USR_01</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Bắt lỗi khi thiếu các trường bắt buộc (email, username, password, fullname, role)</t>
+          <t>Admin tạo tài khoản vai trò Admin thành công</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-Lần lượt gửi payload thiếu: email, ten_dang_nhap, mat_khau, ho_ten, vai_tro</t>
+          <t>POST /api/v1/admin/users {vai_tro: 'Admin', ...}</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Status 422 Unprocessable Entity từ Pydantic Validation Error</t>
+          <t>Status 201 Created, trả về đúng vai_tro='Admin'</t>
         </is>
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity cho tất cả các trường hợp thiếu dữ liệu</t>
+          <t>HTTP 201 Created, tạo tài khoản Admin thành công</t>
         </is>
       </c>
       <c r="J16" s="14" t="inlineStr">
@@ -1796,7 +1740,7 @@
       </c>
       <c r="K16" s="12" t="inlineStr"/>
     </row>
-    <row r="17" ht="45" customHeight="1">
+    <row r="17" ht="42" customHeight="1">
       <c r="A17" s="12" t="n">
         <v>16</v>
       </c>
@@ -1807,39 +1751,37 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_09</t>
+          <t>TC_USR_02</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Bắt lỗi khi vai trò không thuộc danh mục enum hợp lệ</t>
+          <t>Admin tạo tài khoản vai trò HR thành công</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-Payload có vai_tro: 'GiamDocDieuHanh' (ngoài danh mục)</t>
+          <t>POST /api/v1/admin/users {vai_tro: 'HR', ...}</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>Status 422 Unprocessable Entity
-Báo lỗi giá trị vai trò không hợp lệ</t>
+          <t>Status 201 Created, trả về đúng vai_tro='HR'</t>
         </is>
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity chặn giá trị ngoài Enum</t>
+          <t>HTTP 201 Created, tạo tài khoản HR thành công</t>
         </is>
       </c>
       <c r="J17" s="14" t="inlineStr">
@@ -1849,7 +1791,7 @@
       </c>
       <c r="K17" s="12" t="inlineStr"/>
     </row>
-    <row r="18" ht="45" customHeight="1">
+    <row r="18" ht="42" customHeight="1">
       <c r="A18" s="12" t="n">
         <v>17</v>
       </c>
@@ -1860,39 +1802,37 @@
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_10</t>
+          <t>TC_USR_03</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Bắt lỗi khi định dạng email không đúng chuẩn RFC</t>
+          <t>Admin tạo tài khoản vai trò Mentor thành công</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-Payload có email: 'khong-phai-email-hop-le'</t>
+          <t>POST /api/v1/admin/users {vai_tro: 'Mentor', ...}</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Status 422 Unprocessable Entity
-Báo lỗi định dạng email</t>
+          <t>Status 201 Created, trả về đúng vai_tro='Mentor'</t>
         </is>
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>HTTP 422 Unprocessable Entity từ Pydantic EmailStr validator</t>
+          <t>HTTP 201 Created, tạo tài khoản Mentor thành công</t>
         </is>
       </c>
       <c r="J18" s="14" t="inlineStr">
@@ -1902,7 +1842,7 @@
       </c>
       <c r="K18" s="12" t="inlineStr"/>
     </row>
-    <row r="19" ht="45" customHeight="1">
+    <row r="19" ht="42" customHeight="1">
       <c r="A19" s="12" t="n">
         <v>18</v>
       </c>
@@ -1913,38 +1853,37 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_11</t>
+          <t>TC_USR_04</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Chặn người dùng không có quyền Admin tạo tài khoản (HR, Mentor, Thực tập sinh)</t>
+          <t>Admin tạo tài khoản vai trò ThucTapSinh thành công</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-Kèm Bearer Token của HR / Mentor / Thực tập sinh</t>
+          <t>POST /api/v1/admin/users {vai_tro: 'ThucTapSinh', ...}</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>Status 403 Forbidden cho tất cả các vai trò không phải Admin</t>
+          <t>Status 201 Created, trả về đúng vai_tro='ThucTapSinh'</t>
         </is>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>HTTP 403 Forbidden phân quyền RBAC hoạt động chính xác</t>
+          <t>HTTP 201 Created, tạo tài khoản TTS thành công</t>
         </is>
       </c>
       <c r="J19" s="14" t="inlineStr">
@@ -1954,7 +1893,7 @@
       </c>
       <c r="K19" s="12" t="inlineStr"/>
     </row>
-    <row r="20" ht="45" customHeight="1">
+    <row r="20" ht="42" customHeight="1">
       <c r="A20" s="12" t="n">
         <v>19</v>
       </c>
@@ -1965,39 +1904,37 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>TC_USR_12</t>
+          <t>TC_USR_05</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Là admin, tạo tài khoản cho HR, mentor và thực tập sinh</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Chặn người dùng chưa xác thực (không gửi Bearer Token) tạo tài khoản</t>
+          <t>Hỗ trợ payload trường tiếng Anh (username, password, full_name, role)</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>POST /api/v1/admin/users
-(Không gửi header Authorization)</t>
+          <t>POST /api/v1/admin/users {full_name, username, password, role}</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Status 401 Unauthorized
-Detail: 'Không thể xác thực thông tin đăng nhập'</t>
+          <t>Status 201 Created, ánh xạ dữ liệu tiếng Anh mượt mà</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>HTTP 401 Unauthorized chặn truy cập nặc danh</t>
+          <t>HTTP 201 Created tương thích hoàn hảo alias</t>
         </is>
       </c>
       <c r="J20" s="14" t="inlineStr">
@@ -2007,28 +1944,28 @@
       </c>
       <c r="K20" s="12" t="inlineStr"/>
     </row>
-    <row r="21" ht="45" customHeight="1">
+    <row r="21" ht="42" customHeight="1">
       <c r="A21" s="12" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_01</t>
+          <t>TC_USR_06</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Người dùng chưa đăng nhập gọi API nhật ký hoạt động</t>
+          <t>Mật khẩu băm an toàn bằng bcrypt trong DB và không lộ trong response</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
@@ -2038,18 +1975,17 @@
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs
-(Không gửi header Authorization)</t>
+          <t>POST /api/v1/admin/users mang mật khẩu thô</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>Status 401 Unauthorized</t>
+          <t>Status 201 Created; response không lộ password; DB băm bcrypt ($2b$)</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>HTTP 401 Unauthorized đúng cơ chế bảo mật JWT</t>
+          <t>HTTP 201 Created, bảo mật bcrypt an toàn tuyệt đối</t>
         </is>
       </c>
       <c r="J21" s="14" t="inlineStr">
@@ -2059,50 +1995,48 @@
       </c>
       <c r="K21" s="12" t="inlineStr"/>
     </row>
-    <row r="22" ht="45" customHeight="1">
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" s="12" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_02</t>
+          <t>TC_USR_07</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>Chặn người dùng không phải Admin (Thực tập sinh, HR, Mentor) xem nhật ký</t>
+          <t>Bắt lỗi chống trùng lặp tên đăng nhập (username)</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs
-Kèm token của Thực tập sinh, HR, Mentor</t>
+          <t>POST /api/v1/admin/users với ten_dang_nhap đã tồn tại</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Status 403 Forbidden
-Detail: 'Chỉ quản trị viên (Admin) mới có quyền truy cập nhật ký hoạt động'</t>
+          <t>Status 400 Bad Request / 409 Conflict</t>
         </is>
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>HTTP 403 Forbidden chặn vai trò không có quyền xem log hệ thống</t>
+          <t>HTTP 400 Bad Request báo trùng tên đăng nhập</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
@@ -2112,51 +2046,48 @@
       </c>
       <c r="K22" s="12" t="inlineStr"/>
     </row>
-    <row r="23" ht="45" customHeight="1">
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="12" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_03</t>
+          <t>TC_USR_08</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Admin truy vấn danh sách nhật ký hoạt động thành công</t>
+          <t>Bắt lỗi chống trùng lặp địa chỉ email</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs
-(Header: Bearer token Admin)</t>
+          <t>POST /api/v1/admin/users với email đã tồn tại</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Cấu trúc trả về: items, total, page, page_size, total_pages
-Mỗi item có đầy đủ: ma_nhat_ky, endpoint, phuong_thuc, hanh_dong, thoi_gian</t>
+          <t>Status 400 Bad Request / 409 Conflict</t>
         </is>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, đầy đủ metadata phân trang và danh sách nhật ký</t>
+          <t>HTTP 400 Bad Request báo trùng email</t>
         </is>
       </c>
       <c r="J23" s="14" t="inlineStr">
@@ -2166,51 +2097,48 @@
       </c>
       <c r="K23" s="12" t="inlineStr"/>
     </row>
-    <row r="24" ht="45" customHeight="1">
+    <row r="24" ht="42" customHeight="1">
       <c r="A24" s="12" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_04</t>
+          <t>TC_USR_09</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>Phân trang nhật ký (page, page_size), không trùng lặp bản ghi giữa các trang</t>
+          <t>Thiếu trường bắt buộc email</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs?page=1&amp;page_size=2
-và GET /api/v1/admin/audit-logs?page=2&amp;page_size=2</t>
+          <t>POST /api/v1/admin/users thiếu field email</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Trang 1 lấy 2 log, trang 2 lấy 2 log tiếp theo
-Tập ID của trang 1 và trang 2 không giao nhau</t>
+          <t>Status 422 Unprocessable Entity</t>
         </is>
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, thuật toán phân trang hoạt động chuẩn xác</t>
+          <t>HTTP 422 Unprocessable Entity từ Pydantic</t>
         </is>
       </c>
       <c r="J24" s="14" t="inlineStr">
@@ -2220,50 +2148,48 @@
       </c>
       <c r="K24" s="12" t="inlineStr"/>
     </row>
-    <row r="25" ht="45" customHeight="1">
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="12" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_05</t>
+          <t>TC_USR_10</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Tìm kiếm nhật ký theo từ khóa search (trong mô tả, username, endpoint, IP)</t>
+          <t>Thiếu trường bắt buộc ten_dang_nhap (username)</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs?search=Nguyễn+Văn+An
-(Header: Bearer token Admin)</t>
+          <t>POST /api/v1/admin/users thiếu field ten_dang_nhap</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Chỉ trả về các bản ghi log có chứa từ khóa 'Nguyễn Văn An' trong mo_ta/username</t>
+          <t>Status 422 Unprocessable Entity</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, lọc đúng 2 bản ghi chứa từ khóa tìm kiếm</t>
+          <t>HTTP 422 Unprocessable Entity từ Pydantic</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
@@ -2273,49 +2199,48 @@
       </c>
       <c r="K25" s="12" t="inlineStr"/>
     </row>
-    <row r="26" ht="45" customHeight="1">
+    <row r="26" ht="42" customHeight="1">
       <c r="A26" s="12" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_06</t>
+          <t>TC_USR_11</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Bộ lọc nhật ký theo khoảng thời gian tu_ngay và den_ngay</t>
+          <t>Thiếu trường bắt buộc mat_khau (password)</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs?tu_ngay=2026-10-15T00:00:00&amp;den_ngay=2026-10-17T23:59:59</t>
+          <t>POST /api/v1/admin/users thiếu field mat_khau</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Chỉ lấy các bản ghi phát sinh trong khoảng thời gian chỉ định (2 bản ghi)</t>
+          <t>Status 422 Unprocessable Entity</t>
         </is>
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, lọc chính xác theo mốc thời gian ISO</t>
+          <t>HTTP 422 Unprocessable Entity từ Pydantic</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
@@ -2325,49 +2250,48 @@
       </c>
       <c r="K26" s="12" t="inlineStr"/>
     </row>
-    <row r="27" ht="45" customHeight="1">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="12" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_07</t>
+          <t>TC_USR_12</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>Bộ lọc nhật ký theo mã người dùng ma_nguoi_dung</t>
+          <t>Thiếu trường bắt buộc ho_ten (full_name)</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs?ma_nguoi_dung={normal_user.ma_nguoi_dung}</t>
+          <t>POST /api/v1/admin/users thiếu field ho_ten</t>
         </is>
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Chỉ trả về các log phát sinh do user tương ứng thực hiện (TAO_YEU_CAU_HO_TRO)</t>
+          <t>Status 422 Unprocessable Entity</t>
         </is>
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, lọc chuẩn xác theo user ID</t>
+          <t>HTTP 422 Unprocessable Entity từ Pydantic</t>
         </is>
       </c>
       <c r="J27" s="14" t="inlineStr">
@@ -2377,49 +2301,48 @@
       </c>
       <c r="K27" s="12" t="inlineStr"/>
     </row>
-    <row r="28" ht="45" customHeight="1">
+    <row r="28" ht="42" customHeight="1">
       <c r="A28" s="12" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>TC-AuditLogs</t>
+          <t>TC-AdminUser</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>TC_LOG_08</t>
+          <t>TC_USR_13</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
+          <t>Là admin, tạo tài khoản người dùng</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>Bộ lọc kết hợp theo mã hành động và phương thức HTTP</t>
+          <t>Thiếu trường bắt buộc vai_tro (role)</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>GET /api/v1/admin/audit-logs?hanh_dong=CAP_NHAT_NGUOI_DUNG&amp;phuong_thuc=PUT</t>
+          <t>POST /api/v1/admin/users thiếu field vai_tro</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>Status 200 OK
-Lọc chính xác theo cả 2 tiêu chí hanh_dong và phuong_thuc</t>
+          <t>Status 422 Unprocessable Entity</t>
         </is>
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>HTTP 200 OK, trả về đúng bản ghi tương ứng</t>
+          <t>HTTP 422 Unprocessable Entity từ Pydantic</t>
         </is>
       </c>
       <c r="J28" s="14" t="inlineStr">
@@ -2429,57 +2352,1382 @@
       </c>
       <c r="K28" s="12" t="inlineStr"/>
     </row>
-    <row r="29" ht="45" customHeight="1">
+    <row r="29" ht="42" customHeight="1">
       <c r="A29" s="12" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_14</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Bắt lỗi vai trò không thuộc danh mục enum (GiamDocDieuHanh)</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users {vai_tro: 'GiamDocDieuHanh'}</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>Status 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity chặn giá trị ngoài enum</t>
+        </is>
+      </c>
+      <c r="J29" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_15</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Bắt lỗi định dạng email sai chuẩn RFC (khong-phai-email)</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users {email: 'khong-phai-email'}</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>Status 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 422 Unprocessable Entity từ EmailStr</t>
+        </is>
+      </c>
+      <c r="J30" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K30" s="12" t="inlineStr"/>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_16</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Hỗ trợ họ tên tiếng Việt có dấu đầy đủ Unicode UTF-8</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G31" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users {ho_ten: 'Nguyễn Trần Hoàng Đăng Khoa'}</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>Status 201 Created, lưu đúng họ tên có dấu</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created xử lý UTF-8 hoàn hảo</t>
+        </is>
+      </c>
+      <c r="J31" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K31" s="12" t="inlineStr"/>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_17</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>Tài khoản vai trò HR cố tình tạo user -&gt; 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users (Token HR)</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>Status 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden phân quyền RBAC thành công</t>
+        </is>
+      </c>
+      <c r="J32" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr"/>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_18</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>Tài khoản vai trò Mentor cố tình tạo user -&gt; 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users (Token Mentor)</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Status 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden phân quyền RBAC thành công</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K33" s="12" t="inlineStr"/>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_19</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>Tài khoản vai trò ThucTapSinh cố tình tạo user -&gt; 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users (Token ThucTapSinh)</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>Status 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden phân quyền RBAC thành công</t>
+        </is>
+      </c>
+      <c r="J34" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K34" s="12" t="inlineStr"/>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_20</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>Chặn qua header mock X-User-Role: HR -&gt; 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users (Header X-User-Role: HR)</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Status 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden chặn giả mạo vai trò</t>
+        </is>
+      </c>
+      <c r="J35" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr"/>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_21</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>Chưa xác thực token khi tạo user -&gt; 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users (Không gửi Token)</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>Status 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized chặn truy cập nặc danh</t>
+        </is>
+      </c>
+      <c r="J36" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr"/>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>TC-AdminUser</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>TC_USR_22</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, tạo tài khoản người dùng</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Admin xem danh sách người dùng với phân trang và lọc vai trò</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/users?skip=0&amp;limit=10</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, trả về danh sách tài khoản hợp lệ</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK lấy danh sách người dùng thành công</t>
+        </is>
+      </c>
+      <c r="J37" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr"/>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
           <t>TC-AuditLogs</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_01</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Chưa đăng nhập gọi API nhật ký -&gt; 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs (Không gửi Token)</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>Status 401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 401 Unauthorized đúng chuẩn JWT</t>
+        </is>
+      </c>
+      <c r="J38" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K38" s="12" t="inlineStr"/>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_02</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Thực tập sinh không có quyền xem nhật ký -&gt; 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs (Token ThucTapSinh)</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Status 403 Forbidden, detail: 'Chỉ quản trị viên'</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden bảo vệ an toàn nhật ký</t>
+        </is>
+      </c>
+      <c r="J39" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K39" s="12" t="inlineStr"/>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_03</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>HR không có quyền xem nhật ký hệ thống -&gt; 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs (Token HR)</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Status 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden chặn nhân sự xem audit log</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K40" s="12" t="inlineStr"/>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_04</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>Mentor không có quyền xem nhật ký hệ thống -&gt; 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs (Token Mentor)</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>Status 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden chặn mentor xem audit log</t>
+        </is>
+      </c>
+      <c r="J41" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K41" s="12" t="inlineStr"/>
+    </row>
+    <row r="42" ht="42" customHeight="1">
+      <c r="A42" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_05</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E42" s="13" t="inlineStr">
+        <is>
+          <t>Admin xem danh sách nhật ký thành công (200 OK)</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="G42" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs (Token Admin)</t>
+        </is>
+      </c>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, trả về items, total, page, page_size, total_pages</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK đầy đủ dữ liệu nhật ký</t>
+        </is>
+      </c>
+      <c r="J42" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K42" s="12" t="inlineStr"/>
+    </row>
+    <row r="43" ht="42" customHeight="1">
+      <c r="A43" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_06</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E43" s="13" t="inlineStr">
+        <is>
+          <t>Phân trang page 1 và 2 tách biệt, không trùng lặp bản ghi</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G43" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?page=1&amp;page_size=2 và page=2&amp;page_size=2</t>
+        </is>
+      </c>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, tập ID bản ghi giữa 2 trang tách biệt hoàn toàn</t>
+        </is>
+      </c>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK thuật toán phân trang chuẩn xác</t>
+        </is>
+      </c>
+      <c r="J43" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K43" s="12" t="inlineStr"/>
+    </row>
+    <row r="44" ht="42" customHeight="1">
+      <c r="A44" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_07</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>Biên phân trang: page cực lớn trả về danh sách rỗng an toàn</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?page=9999&amp;page_size=20</t>
+        </is>
+      </c>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, items=[] rỗng, không crash lỗi</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK xử lý an toàn biên dữ liệu</t>
+        </is>
+      </c>
+      <c r="J44" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K44" s="12" t="inlineStr"/>
+    </row>
+    <row r="45" ht="42" customHeight="1">
+      <c r="A45" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_08</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>Tìm kiếm nhật ký theo từ khóa trong mô tả (search='Nguyễn Văn An')</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?search=Nguyễn+Văn+An</t>
+        </is>
+      </c>
+      <c r="H45" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, lọc đúng 2 bản ghi chứa tên trong mô tả</t>
+        </is>
+      </c>
+      <c r="I45" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK tìm kiếm từ khóa chính xác</t>
+        </is>
+      </c>
+      <c r="J45" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K45" s="12" t="inlineStr"/>
+    </row>
+    <row r="46" ht="42" customHeight="1">
+      <c r="A46" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>TC_LOG_09</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>Là admin, xem nhật ký hoạt động hệ thống</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>Middleware tự động ghi nhận log chuẩn xác khi phát sinh thao tác dữ liệu</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t>Tìm kiếm nhật ký theo từ khóa endpoint hoặc hành động</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?search=support-requests</t>
+        </is>
+      </c>
+      <c r="H46" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, lọc đúng log có endpoint chứa từ khóa</t>
+        </is>
+      </c>
+      <c r="I46" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK tìm kiếm endpoint chuẩn xác</t>
+        </is>
+      </c>
+      <c r="J46" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K46" s="12" t="inlineStr"/>
+    </row>
+    <row r="47" ht="42" customHeight="1">
+      <c r="A47" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_10</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E47" s="13" t="inlineStr">
+        <is>
+          <t>Bộ lọc nhật ký theo khoảng ngày tu_ngay và den_ngay</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?tu_ngay=2026-10-15&amp;den_ngay=2026-10-17</t>
+        </is>
+      </c>
+      <c r="H47" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, chỉ lấy các bản ghi phát sinh trong khoảng ngày</t>
+        </is>
+      </c>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK lọc theo mốc thời gian chuẩn</t>
+        </is>
+      </c>
+      <c r="J47" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K47" s="12" t="inlineStr"/>
+    </row>
+    <row r="48" ht="42" customHeight="1">
+      <c r="A48" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_11</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>Bộ lọc nhật ký theo mã người dùng ma_nguoi_dung</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G48" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?ma_nguoi_dung={id}</t>
+        </is>
+      </c>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, chỉ trả về hành động do user chỉ định thực hiện</t>
+        </is>
+      </c>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK lọc người dùng chính xác</t>
+        </is>
+      </c>
+      <c r="J48" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K48" s="12" t="inlineStr"/>
+    </row>
+    <row r="49" ht="42" customHeight="1">
+      <c r="A49" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_12</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E49" s="13" t="inlineStr">
+        <is>
+          <t>Bộ lọc kết hợp theo hành động nghiệp vụ và phương thức HTTP</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?hanh_dong=CAP_NHAT_NGUOI_DUNG&amp;phuong_thuc=PUT</t>
+        </is>
+      </c>
+      <c r="H49" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, lọc chính xác theo cả 2 tiêu chí</t>
+        </is>
+      </c>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK kết hợp bộ lọc hoàn hảo</t>
+        </is>
+      </c>
+      <c r="J49" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K49" s="12" t="inlineStr"/>
+    </row>
+    <row r="50" ht="42" customHeight="1">
+      <c r="A50" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_13</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>Sắp xếp danh sách nhật ký theo thời gian giảm dần (DESC)</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs</t>
+        </is>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, bản ghi mới nhất hiển thị trước (thoi_gian 0 &gt;= thoi_gian 1)</t>
+        </is>
+      </c>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK sắp xếp thời gian giảm dần chuẩn</t>
+        </is>
+      </c>
+      <c r="J50" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K50" s="12" t="inlineStr"/>
+    </row>
+    <row r="51" ht="42" customHeight="1">
+      <c r="A51" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_14</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>Middleware tự động ghi log khi phát sinh request POST sửa đổi dữ liệu</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr">
         <is>
           <t>Integration</t>
         </is>
       </c>
-      <c r="G29" s="13" t="inlineStr">
-        <is>
-          <t>Admin gửi POST /api/v1/admin/users tạo người dùng mới với IP giả lập '10.0.1.55'</t>
-        </is>
-      </c>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>Status 201 Created
-Middleware tự động chèn 1 bản ghi mới vào bảng nhat_ky_hoat_dong với đúng endpoint, IP, method, action='TAO_NGUOI_DUNG'</t>
-        </is>
-      </c>
-      <c r="I29" s="13" t="inlineStr">
-        <is>
-          <t>HTTP 201 Created, bảng nhat_ky_hoat_dong tăng 1 bản ghi với dữ liệu chuẩn xác</t>
-        </is>
-      </c>
-      <c r="J29" s="14" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="K29" s="12" t="inlineStr"/>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users tạo người dùng mới</t>
+        </is>
+      </c>
+      <c r="H51" s="13" t="inlineStr">
+        <is>
+          <t>Status 201 Created và bảng nhat_ky_hoat_dong tự động tăng 1 bản ghi</t>
+        </is>
+      </c>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created Middleware tự động ghi log</t>
+        </is>
+      </c>
+      <c r="J51" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K51" s="12" t="inlineStr"/>
+    </row>
+    <row r="52" ht="42" customHeight="1">
+      <c r="A52" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_15</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>Middleware trích xuất đúng IP nguồn từ header X-Forwarded-For</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G52" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users (Header X-Forwarded-For: 203.162.0.100)</t>
+        </is>
+      </c>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>Status 201 Created, dia_chi_ip trong log là '203.162.0.100'</t>
+        </is>
+      </c>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 201 Created trích xuất IP nguồn chuẩn xác</t>
+        </is>
+      </c>
+      <c r="J52" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K52" s="12" t="inlineStr"/>
+    </row>
+    <row r="53" ht="42" customHeight="1">
+      <c r="A53" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_16</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E53" s="13" t="inlineStr">
+        <is>
+          <t>Middleware loại trừ các endpoint kiểm tra sức khỏe /ping</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G53" s="13" t="inlineStr">
+        <is>
+          <t>GET /ping</t>
+        </is>
+      </c>
+      <c r="H53" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, không tạo thêm bản ghi nhật ký mới trong database</t>
+        </is>
+      </c>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK loại trừ endpoint hệ thống chuẩn</t>
+        </is>
+      </c>
+      <c r="J53" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr"/>
+    </row>
+    <row r="54" ht="42" customHeight="1">
+      <c r="A54" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_17</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>Middleware ghi nhận cả thao tác thất bại nghiệp vụ (HTTP 400 Bad Request)</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G54" s="13" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/users gửi trùng username sinh lỗi 400</t>
+        </is>
+      </c>
+      <c r="H54" s="13" t="inlineStr">
+        <is>
+          <t>Status 400 và Middleware vẫn ghi nhận log với mo_ta chứa mã 400</t>
+        </is>
+      </c>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 400 ghi nhận nhật ký thao tác lỗi thành công</t>
+        </is>
+      </c>
+      <c r="J54" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K54" s="12" t="inlineStr"/>
+    </row>
+    <row r="55" ht="42" customHeight="1">
+      <c r="A55" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>TC-AuditLogs</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>TC_LOG_18</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Là admin, xem nhật ký hoạt động</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>Tìm kiếm từ khóa không tồn tại -&gt; trả về total=0 và items=[] an toàn</t>
+        </is>
+      </c>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>GET /api/v1/admin/audit-logs?search=TuKhoaKhongTheTonTai12345</t>
+        </is>
+      </c>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK, total=0, items=[]</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK xử lý tìm kiếm không khớp an toàn</t>
+        </is>
+      </c>
+      <c r="J55" s="14" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="K55" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>